<commit_message>
submittal and tracker updated
</commit_message>
<xml_diff>
--- a/tracker/Project_Control_Tracker.xlsx
+++ b/tracker/Project_Control_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\GC Grocery\4_Active_Jobs\Norcross, GA 1517 Lidl - Ground Up\17. - Claude AI\15170000GR-Norcross-GA---Lidl-US\tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86694A0F-CEF2-424D-B1D8-CF76E8E7DAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93735117-5662-4D5E-B51E-847CDB303717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" firstSheet="13" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="562">
   <si>
     <t>PROJECT INFO</t>
   </si>
@@ -1636,6 +1636,156 @@
   </si>
   <si>
     <t>documents\meeting minutes\OAC\Meeting_Minutes_OAC-001_2026-10-01_Rev1.pdf</t>
+  </si>
+  <si>
+    <t>SUB-001</t>
+  </si>
+  <si>
+    <t>23 0503</t>
+  </si>
+  <si>
+    <t>HVAC Package Rev 0 (Procore 230503-1.0 / Fieldwire PSI-0004) - Lennox RTUs &amp; mini-split, CaptiveAire, ductwork, Greenheck/Titus &amp; Fantech/Airius air distribution, prelim TAB. Reviewer: Make Corrections Noted 9/14 - provide missing EF-1 &amp; air terminal info (addressed in Rev 1). Req'd return = 14-day default; Procore had no due date.</t>
+  </si>
+  <si>
+    <t>Product Data</t>
+  </si>
+  <si>
+    <t>Platinum Air Systems</t>
+  </si>
+  <si>
+    <t>Approved as Noted</t>
+  </si>
+  <si>
+    <t>SUB-001_R1_Original_Procore_Export_2026-10-01.pdf; Submittal-001_Transmittal_Packaged.pdf (package INCLUDED, 659 pp); SUB-001_R0_Reviewed_MakeCorrectionsNoted_2026-09-14.pdf; SUB-001_R1_Reviewed_MakeCorrectionsNoted_2026-09-28.pdf; SUB-001_R1_As-Submitted_PSI-0004_2026-09-22.pdf - folder: documents\submittals\SUB-001 - 230503 HVAC</t>
+  </si>
+  <si>
+    <t>SUB-001-R1</t>
+  </si>
+  <si>
+    <t>HVAC Package Rev 1 (Procore 230503-1.1) - corrections made; EF-1 (SE1-10-440-VG) &amp; Titus air terminals added. Reviewer: Make Corrections Noted 9/28 - OPEN: provide TG-1 per plans and diffuser/register/grille schedule. Procore still Open, ball in court Amy Schoch (Progressive).</t>
+  </si>
+  <si>
+    <t>SUB-002</t>
+  </si>
+  <si>
+    <t>33 4100</t>
+  </si>
+  <si>
+    <t>Stormwater Package Rev 0 (Procore 33 4100-2.0 / Fieldwire PSI-0002) - Hydro International First Defense hydrodynamic separator (ST8), Up-Flo water quality filter (ST5), Southeast Culvert 84in CMP underground detention. Reviewer: CHA Consulting (Christopher Manes) - no response. Req'd return per Fieldwire response due 9/9; Procore has no due date.</t>
+  </si>
+  <si>
+    <t>Coles Construction</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>SUB-002_R0_Original_Procore_Export_2026-10-01.pdf; Submittal-002_Transmittal_Packaged.pdf (package INCLUDED, 62 pp) - folder: documents\submittals\SUB-002 - 334100 Storm Drainage</t>
+  </si>
+  <si>
+    <t>SUB-003</t>
+  </si>
+  <si>
+    <t>Coles Construction (supplier Core &amp; Main)</t>
+  </si>
+  <si>
+    <t>SUB-003_R0_Original_Procore_Export_2026-10-01.pdf; Submittal-003_Transmittal_Packaged.pdf (package INCLUDED, 92 pp) - folder: documents\submittals\SUB-003 - 334100 Site Utilities</t>
+  </si>
+  <si>
+    <t>HDPE Pipe Rev 0 (Procore 33 4100-1.0, Package #1 Site Utilities / Fieldwire PSI-0001) - ADS N-12 ST IB storm pipe (pkg Section 1). Attachment is the full Core &amp; Main site utility package; Procore splits Package #1 into one item per spec section (sanitary = SUB-004). Reviewer: CHA Consulting (Christopher Manes) - no response. Req'd return per Fieldwire response due 9/11; Procore has no due date.</t>
+  </si>
+  <si>
+    <t>SUB-004</t>
+  </si>
+  <si>
+    <t>33 3000</t>
+  </si>
+  <si>
+    <t>Sanitary Sewer Rev 0 (Procore 33 3000-1.0, Package #1 Site Utilities / Fieldwire PSI-0001) - Diamond Sani-21 PVC sewer pipe &amp; fittings, cleanouts, Star Pipe heavy-duty covers, marking tape (pkg Section 2, export pp. 8-19). Same PSI-0001 attachment as SUB-003. Reviewer: CHA Consulting (Christopher Manes) - no response. Req'd return per Fieldwire response due 9/11; Procore has no due date.</t>
+  </si>
+  <si>
+    <t>SUB-004_R0_Original_Procore_Export_2026-10-01.pdf; SUB-004_R0_Sanitary_Section_Only.pdf; Submittal-004_Transmittal_Packaged.pdf (package INCLUDED, 92 pp) - folder: documents\submittals\SUB-004 - 333000 Sanitary Sewer</t>
+  </si>
+  <si>
+    <t>SUB-005</t>
+  </si>
+  <si>
+    <t>33 1000</t>
+  </si>
+  <si>
+    <t>Domestic Water &amp; Irrigation Rev 0 (Procore 33 1000-1.0, Package #1 Site Utilities / Fieldwire PSI-0001) - PVC pressure pipe &amp; DI fittings, 2in tap assemblies (Smith-Blair 313, Ford Meter Box), 2in DCV (Wilkins 950XLT), irrigation, 2in RPZ (Wilkins 975XL2) (pkg Section 3, export pp. 20-53). Same PSI-0001 attachment as SUB-003/004. Reviewer: CHA Consulting (Christopher Manes) - no response. Req'd return per Fieldwire response due 9/11; Procore has no due date.</t>
+  </si>
+  <si>
+    <t>SUB-005_R0_Original_Procore_Export_2026-10-01.pdf; SUB-005_R0_Domestic_Water_Section_Only.pdf; Submittal-005_Transmittal_Packaged.pdf (package INCLUDED, 92 pp) - folder: documents\submittals\SUB-005 - 331000 Domestic Water</t>
+  </si>
+  <si>
+    <t>SUB-006</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>Fire Main Rev 0 (Procore 33-1.0, Package #1 Site Utilities) - U.S. Pipe Tyton DI pipe &amp; fittings, tapping sleeve, M&amp;H 129 hydrant, 8in DCDA BFP vault (Wilkins 350ASTDA), 8in PIV, 8in gate valve (PSI-0001 pkg Section 4, export pp. 54-91). FLAG: Procore item has NO ATTACHMENT (cover only) and spec is division-level '33 - Utilities' - confirm CHA has the fire main cut sheets. Reviewer: CHA Consulting (Christopher Manes) - no response. Req'd return per Fieldwire response due 9/11.</t>
+  </si>
+  <si>
+    <t>SUB-006_R0_Procore_Cover_Only_2026-10-01.pdf (Procore item has NO attachment); SUB-006_R0_Fire_Main_Section_REFERENCE_from_PSI-0001.pdf (from SUB-003 copy); Submittal-006_Transmittal_Packaged.pdf (42 pp) - folder: documents\submittals\SUB-006 - 33 Fire Main</t>
+  </si>
+  <si>
+    <t>SUB-007</t>
+  </si>
+  <si>
+    <t>22 (22 1119)</t>
+  </si>
+  <si>
+    <t>Plumbing Package Rev 0 (Procore 22-1.0, Package #2 Plumbing / Fieldwire PSI-0003) - fixtures (DF, L, WC, SK-1/2/3), hydrants, floor drains/sinks, PRV, EWH-1, gas meter. Procore CLOSED. Reviewer (Progressive, bizons 9/25): Make Corrections Noted - OPEN: SK-3 replace Elkay SS8354LR4 with Elkay 14-3C16X20-L-18X per CCD 01 (05/28/2026). Returned 14 days after 9/11 due date.</t>
+  </si>
+  <si>
+    <t>Golden Hands Plumbing (supplier Cowan Supply)</t>
+  </si>
+  <si>
+    <t>SUB-007_R0_Original_Procore_Export_2026-10-01.pdf; SUB-007_R0_Reviewed_MakeCorrectionsNoted_2026-09-25.pdf; SUB-007_R0_As-Submitted_PSI-0003_2026-09-03.pdf; Submittal-007_Transmittal_Packaged.pdf (package INCLUDED, 217 pp) - folder: documents\submittals\SUB-007 - 22 Plumbing</t>
+  </si>
+  <si>
+    <t>SUB-008</t>
+  </si>
+  <si>
+    <t>None (Procore '1 - Default')</t>
+  </si>
+  <si>
+    <t>CCTV Submittal Rev 0 (Procore 1-3.0 / Fieldwire PSI-0007) - off-site traffic signal Gwinnett Co. TS-082, Jimmy Carter Blvd @ Shelby Dr: AXIS Q6086-E PTZ camera, Major Custom Cable CAT6 100ft, DITEK DTK-MRJPOES surge protector, AXIS TQ5001-E mount (Utilicom quote 62085). No spec section assigned. Reviewer: CHA Consulting (Christopher Manes) - no response; confirm whether Gwinnett DOT review also required. Req'd return per Fieldwire response due 9/25.</t>
+  </si>
+  <si>
+    <t>R.J. Haynie &amp; Associates (supplier Utilicom Supply Associates)</t>
+  </si>
+  <si>
+    <t>SUB-008_R0_Original_Procore_Export_2026-10-01.pdf; Submittal-008_Transmittal_Packaged.pdf (package INCLUDED, 18 pp) - folder: documents\submittals\SUB-008 - CCTV Traffic Signal</t>
+  </si>
+  <si>
+    <t>SUB-009</t>
+  </si>
+  <si>
+    <t>Mast Arm Pole Shop Drawings #1-#3 Rev 0 (Procore 1-2.0 / Fieldwire PSI-0006) - off-site traffic signal Gwinnett Co. TS-082, Jimmy Carter Blvd @ Shelby Dr: Valmont GA672263P1 (2 sheets, GA PE sealed 8/31) Poles B (22ft, 65+55ft arms) &amp; C (30ft, 55+55ft arms) + orientation sketch. FLAG: foundation callout (3ft dia x 14.5ft, (8) #10) is an unsigned annotation, not on sealed dwg - verify. Reviewer: CHA Consulting (Christopher Manes) - no response; confirm Gwinnett DOT review. Req'd return per Fieldwire due 9/25.</t>
+  </si>
+  <si>
+    <t>Shop Drawing</t>
+  </si>
+  <si>
+    <t>R.J. Haynie &amp; Associates (Valmont via DOT Lighting / Traffic &amp; Lighting Corp)</t>
+  </si>
+  <si>
+    <t>SUB-009_R0_Original_Procore_Export_2026-10-01.pdf; Submittal-009_Transmittal_Packaged.pdf (package INCLUDED, 6 pp) - folder: documents\submittals\SUB-009 - Mast Arm Poles</t>
+  </si>
+  <si>
+    <t>SUB-010</t>
+  </si>
+  <si>
+    <t>Mast Arm Pole Submittals Rev 0 (Procore 1-1.0 / Fieldwire PSI-0005) - Valmont structural calcs, Order 672263-P1 (94 pp), Poles B (P22 M65/M55) &amp; C (P30 M55/M55), AASHTO 2015, 115 mph - off-site signal Gwinnett Co. TS-082. Related to SUB-009 shop dwgs. FLAG: calcs give foundation reactions only, no foundation design; PE seal is image stamp, not digitally signed. Reviewer: CHA Consulting (Christopher Manes) - no response. Req'd return per Fieldwire due 9/25.</t>
+  </si>
+  <si>
+    <t>R.J. Haynie &amp; Associates (Valmont Industries)</t>
+  </si>
+  <si>
+    <t>SUB-010_R0_Original_Procore_Export_2026-10-01.pdf; Submittal-010_Transmittal_Packaged.pdf (package INCLUDED, 99 pp) - folder: documents\submittals\SUB-010 - Mast Arm Pole Calcs</t>
   </si>
 </sst>
 </file>
@@ -1782,7 +1932,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1816,6 +1966,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18161,7 +18312,7 @@
       </c>
       <c r="C15" s="4">
         <f>COUNTIFS('Submittal Log'!G2:G299,"&lt;&gt;",'Submittal Log'!I2:I299,"")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
@@ -18461,7 +18612,7 @@
       </c>
       <c r="C52" s="4">
         <f ca="1">COUNTIF('Submittal Log'!P2:P299,"&gt;=14")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.25">
@@ -24423,13 +24574,49 @@
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K2" t="str">
+      <c r="A2" t="s">
+        <v>512</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>513</v>
+      </c>
+      <c r="C2" t="s">
+        <v>514</v>
+      </c>
+      <c r="D2" t="s">
+        <v>515</v>
+      </c>
+      <c r="E2" t="s">
+        <v>516</v>
+      </c>
+      <c r="F2" s="25">
+        <v>46268</v>
+      </c>
+      <c r="G2" s="25">
+        <v>46274</v>
+      </c>
+      <c r="H2" s="25">
+        <v>46288</v>
+      </c>
+      <c r="I2" s="25">
+        <v>46289</v>
+      </c>
+      <c r="J2" t="s">
+        <v>517</v>
+      </c>
+      <c r="K2">
         <f t="shared" ref="K2:K65" ca="1" si="0">IF(A2="","",IF(I2&lt;&gt;"",I2-G2,IF(G2&lt;&gt;"",TODAY()-G2,"")))</f>
-        <v/>
-      </c>
-      <c r="O2" s="13" t="str">
+        <v>15</v>
+      </c>
+      <c r="M2" t="s">
+        <v>518</v>
+      </c>
+      <c r="N2" t="s">
+        <v>274</v>
+      </c>
+      <c r="O2" s="13">
         <f t="shared" ref="O2:O65" si="1">IF(A2="","",MAX(F2+0,G2+0,H2+0,I2+0))</f>
-        <v/>
+        <v>46289</v>
       </c>
       <c r="P2" t="str">
         <f t="shared" ref="P2:P65" ca="1" si="2">IF(A2="","",IF(OR(J2="Approved",J2="Approved as Noted"),"",TODAY()-O2))</f>
@@ -24437,13 +24624,49 @@
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K3" t="str">
+      <c r="A3" t="s">
+        <v>519</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>513</v>
+      </c>
+      <c r="C3" t="s">
+        <v>520</v>
+      </c>
+      <c r="D3" t="s">
+        <v>515</v>
+      </c>
+      <c r="E3" t="s">
+        <v>516</v>
+      </c>
+      <c r="F3" s="25">
+        <v>46287</v>
+      </c>
+      <c r="G3" s="25">
+        <v>46287</v>
+      </c>
+      <c r="H3" s="25">
+        <v>46309</v>
+      </c>
+      <c r="I3" s="25">
+        <v>46293</v>
+      </c>
+      <c r="J3" t="s">
+        <v>517</v>
+      </c>
+      <c r="K3">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O3" s="13" t="str">
+        <v>6</v>
+      </c>
+      <c r="M3" t="s">
+        <v>518</v>
+      </c>
+      <c r="N3" t="s">
+        <v>274</v>
+      </c>
+      <c r="O3" s="13">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46309</v>
       </c>
       <c r="P3" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -24451,83 +24674,284 @@
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K4" t="str">
+      <c r="A4" t="s">
+        <v>521</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>522</v>
+      </c>
+      <c r="C4" t="s">
+        <v>523</v>
+      </c>
+      <c r="D4" t="s">
+        <v>515</v>
+      </c>
+      <c r="E4" t="s">
+        <v>524</v>
+      </c>
+      <c r="F4" s="25">
+        <v>46260</v>
+      </c>
+      <c r="G4" s="25">
+        <v>46260</v>
+      </c>
+      <c r="H4" s="25">
+        <v>46274</v>
+      </c>
+      <c r="J4" t="s">
+        <v>525</v>
+      </c>
+      <c r="K4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O4" s="13" t="str">
+        <v>36</v>
+      </c>
+      <c r="M4" t="s">
+        <v>526</v>
+      </c>
+      <c r="N4" t="s">
+        <v>274</v>
+      </c>
+      <c r="O4" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P4" t="str">
+        <v>46274</v>
+      </c>
+      <c r="P4">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K5" t="str">
+      <c r="A5" t="s">
+        <v>527</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>522</v>
+      </c>
+      <c r="C5" t="s">
+        <v>530</v>
+      </c>
+      <c r="D5" t="s">
+        <v>515</v>
+      </c>
+      <c r="E5" t="s">
+        <v>528</v>
+      </c>
+      <c r="F5" s="25">
+        <v>46260</v>
+      </c>
+      <c r="G5" s="25">
+        <v>46260</v>
+      </c>
+      <c r="H5" s="25">
+        <v>46276</v>
+      </c>
+      <c r="J5" t="s">
+        <v>525</v>
+      </c>
+      <c r="K5">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O5" s="13" t="str">
+        <v>36</v>
+      </c>
+      <c r="M5" t="s">
+        <v>529</v>
+      </c>
+      <c r="N5" t="s">
+        <v>274</v>
+      </c>
+      <c r="O5" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P5" t="str">
+        <v>46276</v>
+      </c>
+      <c r="P5">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K6" t="str">
+      <c r="A6" t="s">
+        <v>531</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>532</v>
+      </c>
+      <c r="C6" t="s">
+        <v>533</v>
+      </c>
+      <c r="D6" t="s">
+        <v>515</v>
+      </c>
+      <c r="E6" t="s">
+        <v>528</v>
+      </c>
+      <c r="F6" s="25">
+        <v>46260</v>
+      </c>
+      <c r="G6" s="25">
+        <v>46260</v>
+      </c>
+      <c r="H6" s="25">
+        <v>46276</v>
+      </c>
+      <c r="J6" t="s">
+        <v>525</v>
+      </c>
+      <c r="K6">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O6" s="13" t="str">
+        <v>36</v>
+      </c>
+      <c r="M6" t="s">
+        <v>534</v>
+      </c>
+      <c r="N6" t="s">
+        <v>274</v>
+      </c>
+      <c r="O6" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P6" t="str">
+        <v>46276</v>
+      </c>
+      <c r="P6">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K7" t="str">
+      <c r="A7" t="s">
+        <v>535</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>536</v>
+      </c>
+      <c r="C7" t="s">
+        <v>537</v>
+      </c>
+      <c r="D7" t="s">
+        <v>515</v>
+      </c>
+      <c r="E7" t="s">
+        <v>528</v>
+      </c>
+      <c r="F7" s="25">
+        <v>46260</v>
+      </c>
+      <c r="G7" s="25">
+        <v>46260</v>
+      </c>
+      <c r="H7" s="25">
+        <v>46276</v>
+      </c>
+      <c r="J7" t="s">
+        <v>525</v>
+      </c>
+      <c r="K7">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O7" s="13" t="str">
+        <v>36</v>
+      </c>
+      <c r="M7" t="s">
+        <v>538</v>
+      </c>
+      <c r="N7" t="s">
+        <v>274</v>
+      </c>
+      <c r="O7" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P7" t="str">
+        <v>46276</v>
+      </c>
+      <c r="P7">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K8" t="str">
+      <c r="A8" t="s">
+        <v>539</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>540</v>
+      </c>
+      <c r="C8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D8" t="s">
+        <v>515</v>
+      </c>
+      <c r="E8" t="s">
+        <v>528</v>
+      </c>
+      <c r="F8" s="25">
+        <v>46260</v>
+      </c>
+      <c r="G8" s="25">
+        <v>46260</v>
+      </c>
+      <c r="H8" s="25">
+        <v>46276</v>
+      </c>
+      <c r="J8" t="s">
+        <v>525</v>
+      </c>
+      <c r="K8">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O8" s="13" t="str">
+        <v>36</v>
+      </c>
+      <c r="M8" t="s">
+        <v>542</v>
+      </c>
+      <c r="N8" t="s">
+        <v>274</v>
+      </c>
+      <c r="O8" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P8" t="str">
+        <v>46276</v>
+      </c>
+      <c r="P8">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K9" t="str">
+      <c r="A9" t="s">
+        <v>543</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>544</v>
+      </c>
+      <c r="C9" t="s">
+        <v>545</v>
+      </c>
+      <c r="D9" t="s">
+        <v>515</v>
+      </c>
+      <c r="E9" t="s">
+        <v>546</v>
+      </c>
+      <c r="F9" s="25">
+        <v>46260</v>
+      </c>
+      <c r="G9" s="25">
+        <v>46268</v>
+      </c>
+      <c r="H9" s="25">
+        <v>46276</v>
+      </c>
+      <c r="I9" s="25">
+        <v>46290</v>
+      </c>
+      <c r="J9" t="s">
+        <v>517</v>
+      </c>
+      <c r="K9">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O9" s="13" t="str">
+        <v>22</v>
+      </c>
+      <c r="M9" t="s">
+        <v>547</v>
+      </c>
+      <c r="N9" t="s">
+        <v>274</v>
+      </c>
+      <c r="O9" s="13">
         <f t="shared" si="1"/>
-        <v/>
+        <v>46290</v>
       </c>
       <c r="P9" t="str">
         <f t="shared" ca="1" si="2"/>
@@ -24535,45 +24959,144 @@
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K10" t="str">
+      <c r="A10" t="s">
+        <v>548</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>549</v>
+      </c>
+      <c r="C10" t="s">
+        <v>550</v>
+      </c>
+      <c r="D10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E10" t="s">
+        <v>551</v>
+      </c>
+      <c r="F10" s="25">
+        <v>46265</v>
+      </c>
+      <c r="G10" s="25">
+        <v>46283</v>
+      </c>
+      <c r="H10" s="25">
+        <v>46290</v>
+      </c>
+      <c r="J10" t="s">
+        <v>525</v>
+      </c>
+      <c r="K10">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O10" s="13" t="str">
+        <v>13</v>
+      </c>
+      <c r="M10" t="s">
+        <v>552</v>
+      </c>
+      <c r="N10" t="s">
+        <v>274</v>
+      </c>
+      <c r="O10" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P10" t="str">
+        <v>46290</v>
+      </c>
+      <c r="P10">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K11" t="str">
+      <c r="A11" t="s">
+        <v>553</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>549</v>
+      </c>
+      <c r="C11" t="s">
+        <v>554</v>
+      </c>
+      <c r="D11" t="s">
+        <v>555</v>
+      </c>
+      <c r="E11" t="s">
+        <v>556</v>
+      </c>
+      <c r="F11" s="25">
+        <v>46265</v>
+      </c>
+      <c r="G11" s="25">
+        <v>46283</v>
+      </c>
+      <c r="H11" s="25">
+        <v>46290</v>
+      </c>
+      <c r="J11" t="s">
+        <v>525</v>
+      </c>
+      <c r="K11">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O11" s="13" t="str">
+        <v>13</v>
+      </c>
+      <c r="M11" t="s">
+        <v>557</v>
+      </c>
+      <c r="N11" t="s">
+        <v>274</v>
+      </c>
+      <c r="O11" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P11" t="str">
+        <v>46290</v>
+      </c>
+      <c r="P11">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="K12" t="str">
+      <c r="A12" t="s">
+        <v>558</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>549</v>
+      </c>
+      <c r="C12" t="s">
+        <v>559</v>
+      </c>
+      <c r="D12" t="s">
+        <v>515</v>
+      </c>
+      <c r="E12" t="s">
+        <v>560</v>
+      </c>
+      <c r="F12" s="25">
+        <v>46265</v>
+      </c>
+      <c r="G12" s="25">
+        <v>46283</v>
+      </c>
+      <c r="H12" s="25">
+        <v>46290</v>
+      </c>
+      <c r="J12" t="s">
+        <v>525</v>
+      </c>
+      <c r="K12">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-      <c r="O12" s="13" t="str">
+        <v>13</v>
+      </c>
+      <c r="M12" t="s">
+        <v>561</v>
+      </c>
+      <c r="N12" t="s">
+        <v>274</v>
+      </c>
+      <c r="O12" s="13">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="P12" t="str">
+        <v>46290</v>
+      </c>
+      <c r="P12">
         <f t="shared" ca="1" si="2"/>
-        <v/>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Change Order 1 and 2 creation
</commit_message>
<xml_diff>
--- a/tracker/Project_Control_Tracker.xlsx
+++ b/tracker/Project_Control_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\GC Grocery\4_Active_Jobs\Norcross, GA 1517 Lidl - Ground Up\17. - Claude AI\15170000GR-Norcross-GA---Lidl-US\tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93735117-5662-4D5E-B51E-847CDB303717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95BC9F3-88BD-4A5A-9911-60C6C5875E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" tabRatio="500" firstSheet="13" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1215" yWindow="4035" windowWidth="28800" windowHeight="17145" tabRatio="500" firstSheet="16" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Info" sheetId="1" r:id="rId1"/>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="580">
   <si>
     <t>PROJECT INFO</t>
   </si>
@@ -1786,6 +1786,60 @@
   </si>
   <si>
     <t>SUB-010_R0_Original_Procore_Export_2026-10-01.pdf; Submittal-010_Transmittal_Packaged.pdf (package INCLUDED, 99 pp) - folder: documents\submittals\SUB-010 - Mast Arm Pole Calcs</t>
+  </si>
+  <si>
+    <t>PCO-001</t>
+  </si>
+  <si>
+    <t>Owner Request</t>
+  </si>
+  <si>
+    <t>Earthwork/Site Utilities, Roofing, Low Voltage, Metal Panels, Plumbing, Rooftop Screens, Doors/Frames/Hardware</t>
+  </si>
+  <si>
+    <t>OCO-01</t>
+  </si>
+  <si>
+    <t>Base bid material/fuel price escalation true-up (Q1 2026 bid to July 2026 award); 5% OH&amp;P</t>
+  </si>
+  <si>
+    <t>CO #01 - OCO Package - Pricing Escalation Rebalance.pdf (incl. PSI PCO-001 cost breakdown); 22_GC_CO_Template - CO01 rev1.xlsx; OCO #01 - Email Backup (7/29-8/3/2026)</t>
+  </si>
+  <si>
+    <t>SCO-LOG-001</t>
+  </si>
+  <si>
+    <t>CO-02 Asbestos abatement (Georgia Environmental): Main Event Hall ACM floor mastic/carpet glue/carpet + ACM roofing mastic at 8 roof vents</t>
+  </si>
+  <si>
+    <t>PCO-002 / OCO-02</t>
+  </si>
+  <si>
+    <t>PCO-002</t>
+  </si>
+  <si>
+    <t>Allowance #01 - building demolition + ACM abatement; $224,903.34 drawn from $225,000 Demolition Allowance ($96.66 remaining); net $0 to Contract Sum; 9.8% GC OH&amp;P</t>
+  </si>
+  <si>
+    <t>OCO-02</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Luis Marcelino, General Manager</t>
+  </si>
+  <si>
+    <t>Lidl #1517 - Change Order #2 - Asbestos Abatement.pdf; SCO - Coles Construction CO-02.xlsx</t>
+  </si>
+  <si>
+    <t>Valid change: Subcontract No. 7 (8/4/2026) Exhibit A covers selective/building demolition but no asbestos/ACM abatement, and PSI's bid (exclusion h) excludes asbestos abatement. ACM black floor mastic and roof penetration cement are confirmed in Owner's NOVA pre-demolition ACM survey (3/18/2021). Sub O&amp;P 10% = prime contract 4.2 sub cap. Optional $5,500 debris line excluded (debris to be cleared before mobilization). Additional unsampled roof/mirror glue ACM to come as a separate SCO. Approved contingent on Lidl executing CO #02.</t>
+  </si>
+  <si>
+    <t>CO #02 - OCO Package - Building Demolition &amp; Abatement.pdf; Lidl 1517 Demolition Scope.pdf (Cole's demo proposal $148,400); SCO - Coles Construction CO-02.xlsx; Lidl #1517 - Change Order #2 - Asbestos Abatement.pdf (Cole's CO-02 / SCO-LOG-001); 22_GC_CO_Template - CO02.xlsx</t>
+  </si>
+  <si>
+    <t>Demolition (Building &amp; Site), Asbestos Abatement</t>
   </si>
 </sst>
 </file>
@@ -18336,7 +18390,7 @@
       </c>
       <c r="C18" s="4">
         <f>COUNTIF('Change Order Log'!J2:J299,"Pending")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
@@ -18378,7 +18432,7 @@
       </c>
       <c r="C23" s="17">
         <f>SUMIFS('Subcontractor CO Log'!N2:N299,'Subcontractor CO Log'!K2:K299,"Approved")</f>
-        <v>0</v>
+        <v>56430</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.25">
@@ -18621,7 +18675,7 @@
       </c>
       <c r="C53" s="4">
         <f ca="1">COUNTIF('Change Order Log'!Q2:Q299,"&gt;=14")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
@@ -29213,31 +29267,97 @@
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="M2" t="str">
+      <c r="A2" t="s">
+        <v>562</v>
+      </c>
+      <c r="B2" s="25">
+        <v>46254</v>
+      </c>
+      <c r="C2" t="s">
+        <v>566</v>
+      </c>
+      <c r="D2" t="s">
+        <v>563</v>
+      </c>
+      <c r="E2" t="s">
+        <v>564</v>
+      </c>
+      <c r="H2">
+        <v>99986.52</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s">
+        <v>525</v>
+      </c>
+      <c r="M2">
         <f>IF(A2="","",SUMIFS(H$2:H2,J$2:J2,"Approved"))</f>
-        <v/>
-      </c>
-      <c r="P2" s="13" t="str">
+        <v>0</v>
+      </c>
+      <c r="N2" t="s">
+        <v>567</v>
+      </c>
+      <c r="O2" t="s">
+        <v>274</v>
+      </c>
+      <c r="P2" s="13">
         <f t="shared" ref="P2:P65" si="0">IF(A2="","",MAX(B2+0,K2+0,L2+0))</f>
-        <v/>
-      </c>
-      <c r="Q2" t="str">
+        <v>46254</v>
+      </c>
+      <c r="Q2">
         <f t="shared" ref="Q2:Q65" ca="1" si="1">IF(A2="","",IF(OR(J2="Approved",J2="Rejected",J2="Void"),"",TODAY()-P2))</f>
-        <v/>
+        <v>42</v>
+      </c>
+      <c r="R2" t="s">
+        <v>565</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="M3" t="str">
+      <c r="A3" t="s">
+        <v>571</v>
+      </c>
+      <c r="B3" s="25">
+        <v>46259</v>
+      </c>
+      <c r="C3" t="s">
+        <v>572</v>
+      </c>
+      <c r="D3" t="s">
+        <v>563</v>
+      </c>
+      <c r="E3" t="s">
+        <v>579</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s">
+        <v>525</v>
+      </c>
+      <c r="M3">
         <f>IF(A3="","",SUMIFS(H$2:H3,J$2:J3,"Approved"))</f>
-        <v/>
-      </c>
-      <c r="P3" s="13" t="str">
+        <v>0</v>
+      </c>
+      <c r="N3" t="s">
+        <v>578</v>
+      </c>
+      <c r="O3" t="s">
+        <v>274</v>
+      </c>
+      <c r="P3" s="13">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="Q3" t="str">
+        <v>46259</v>
+      </c>
+      <c r="Q3">
         <f t="shared" ca="1" si="1"/>
-        <v/>
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -33490,13 +33610,58 @@
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="O2" t="str">
+      <c r="A2" t="s">
+        <v>568</v>
+      </c>
+      <c r="B2" s="25">
+        <v>46257</v>
+      </c>
+      <c r="C2" t="s">
+        <v>510</v>
+      </c>
+      <c r="D2">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>569</v>
+      </c>
+      <c r="F2">
+        <v>56430</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>570</v>
+      </c>
+      <c r="J2" t="s">
+        <v>577</v>
+      </c>
+      <c r="K2" t="s">
+        <v>574</v>
+      </c>
+      <c r="L2" s="25">
+        <v>46296</v>
+      </c>
+      <c r="M2" t="s">
+        <v>575</v>
+      </c>
+      <c r="N2">
+        <v>56430</v>
+      </c>
+      <c r="O2">
         <f>IF(C2="","",SUMIFS($N$2:N2,$C$2:C2,C2,$K$2:K2,"Approved"))</f>
-        <v/>
-      </c>
-      <c r="R2" s="13" t="str">
+        <v>56430</v>
+      </c>
+      <c r="P2" t="s">
+        <v>576</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>274</v>
+      </c>
+      <c r="R2" s="13">
         <f t="shared" ref="R2:R65" si="0">IF(C2="","",MAX(B2+0,L2+0))</f>
-        <v/>
+        <v>46296</v>
       </c>
       <c r="S2" t="str">
         <f t="shared" ref="S2:S65" ca="1" si="1">IF(C2="","",IF(OR(K2="Approved",K2="Rejected",K2="Void"),"",TODAY()-R2))</f>

</xml_diff>

<commit_message>
CCD 1 and 2 Take Off
</commit_message>
<xml_diff>
--- a/tracker/Project_Control_Tracker.xlsx
+++ b/tracker/Project_Control_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\GC Grocery\4_Active_Jobs\Norcross, GA 1517 Lidl - Ground Up\17. - Claude AI\15170000GR-Norcross-GA---Lidl-US\tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95BC9F3-88BD-4A5A-9911-60C6C5875E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7B48CE0-B4D4-44E3-BC8F-685381009B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1215" yWindow="4035" windowWidth="28800" windowHeight="17145" tabRatio="500" firstSheet="16" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="3210" windowWidth="28800" windowHeight="17145" tabRatio="500" firstSheet="16" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Info" sheetId="1" r:id="rId1"/>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="610">
   <si>
     <t>PROJECT INFO</t>
   </si>
@@ -1840,6 +1840,96 @@
   </si>
   <si>
     <t>Demolition (Building &amp; Site), Asbestos Abatement</t>
+  </si>
+  <si>
+    <t>E101</t>
+  </si>
+  <si>
+    <t>Ground Floor - Electrical Power Plan</t>
+  </si>
+  <si>
+    <t>Electrical</t>
+  </si>
+  <si>
+    <t>2025-12-18 — Issued for Bid (Bid Set, Permit Cycle 2)</t>
+  </si>
+  <si>
+    <t>2026-01-14 — Permit Cycle 3 (not in Bid Set; no narrative)</t>
+  </si>
+  <si>
+    <t>2026-05-28 — CCD 01: undershelf lighting power, refrig/freezer layout, produce power poles, ADA scooter power relocated</t>
+  </si>
+  <si>
+    <t>2026-07-30 — CCD 02: digital sign power, 2 receptacles on LC1-38 (Vestibule), keynote 22</t>
+  </si>
+  <si>
+    <t>Current</t>
+  </si>
+  <si>
+    <t>Lidl 1517 - E-DWGs_Bid Set.pdf; E-DWGs_CCD1.pdf; E-DWGs_CCD2.pdf; CCD2_Comparison_QTO.pdf</t>
+  </si>
+  <si>
+    <t>E300</t>
+  </si>
+  <si>
+    <t>Enlarged Electrical Drawings (Bakery / Technical)</t>
+  </si>
+  <si>
+    <t>2026-07-30 — CCD 02: oven keynote revised to 2x NEMA 15-60R (lower) + 2x 15-50R (upper)</t>
+  </si>
+  <si>
+    <t>Lidl 1517 - E-DWGs_Bid Set.pdf; E-DWGs_CCD2.pdf; CCD2_Comparison_QTO.pdf</t>
+  </si>
+  <si>
+    <t>E301</t>
+  </si>
+  <si>
+    <t>Enlarged Electrical Drawings (Checkout / Cooler-Freezer)</t>
+  </si>
+  <si>
+    <t>2026-05-28 — CCD 01: freezer layout &amp; connections, cooler layout added, checkout power updated</t>
+  </si>
+  <si>
+    <t>2026-07-30 — CCD 02: digital sign power, 2 receptacles on LC1-40 (checkout storefront), keynote 19</t>
+  </si>
+  <si>
+    <t>E501</t>
+  </si>
+  <si>
+    <t>Electrical Panel Schedules</t>
+  </si>
+  <si>
+    <t>2026-05-28 — CCD 01: step-down transformer breakers; bakery oven breakers 20A to 60A/3P</t>
+  </si>
+  <si>
+    <t>2026-07-30 — CCD 02: upper ovens 50A/3P (BK1-13, 25), lower 60A/3P (BK1-19, 31); BK1 57.8 kVA</t>
+  </si>
+  <si>
+    <t>E502</t>
+  </si>
+  <si>
+    <t>2026-05-28 — CCD 01: LA2 panel schedule updated</t>
+  </si>
+  <si>
+    <t>2026-07-30 — CCD 02: LC1-38 / LC1-40 spares become Digital Signage, 720 VA each</t>
+  </si>
+  <si>
+    <t>T101</t>
+  </si>
+  <si>
+    <t>Ground Floor - Technology Plan</t>
+  </si>
+  <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>2026-05-28 — CCD 01: checkout data locations updated; hand hole shifted</t>
+  </si>
+  <si>
+    <t>2026-07-30 — CCD 02: 3 data outlets for digital signs, keynote 30 (vestibule outlet not clouded)</t>
+  </si>
+  <si>
+    <t>Lidl 1517 - T-DWGs_Bid Set.pdf; T-DWGs_CCD1.pdf; T101-CCD2.pdf; CCD2_Comparison_QTO.pdf</t>
   </si>
 </sst>
 </file>
@@ -17336,6 +17426,207 @@
         <v>226</v>
       </c>
     </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>580</v>
+      </c>
+      <c r="B5" t="s">
+        <v>581</v>
+      </c>
+      <c r="C5" t="s">
+        <v>582</v>
+      </c>
+      <c r="D5" t="s">
+        <v>583</v>
+      </c>
+      <c r="E5" t="s">
+        <v>584</v>
+      </c>
+      <c r="F5" t="s">
+        <v>585</v>
+      </c>
+      <c r="G5" t="s">
+        <v>586</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+      <c r="K5" s="25">
+        <v>46233</v>
+      </c>
+      <c r="L5" t="s">
+        <v>587</v>
+      </c>
+      <c r="M5" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>589</v>
+      </c>
+      <c r="B6" t="s">
+        <v>590</v>
+      </c>
+      <c r="C6" t="s">
+        <v>582</v>
+      </c>
+      <c r="D6" t="s">
+        <v>583</v>
+      </c>
+      <c r="E6" t="s">
+        <v>591</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" s="25">
+        <v>46233</v>
+      </c>
+      <c r="L6" t="s">
+        <v>587</v>
+      </c>
+      <c r="M6" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>593</v>
+      </c>
+      <c r="B7" t="s">
+        <v>594</v>
+      </c>
+      <c r="C7" t="s">
+        <v>582</v>
+      </c>
+      <c r="D7" t="s">
+        <v>583</v>
+      </c>
+      <c r="E7" t="s">
+        <v>584</v>
+      </c>
+      <c r="F7" t="s">
+        <v>595</v>
+      </c>
+      <c r="G7" t="s">
+        <v>596</v>
+      </c>
+      <c r="J7">
+        <v>3</v>
+      </c>
+      <c r="K7" s="25">
+        <v>46233</v>
+      </c>
+      <c r="L7" t="s">
+        <v>587</v>
+      </c>
+      <c r="M7" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>597</v>
+      </c>
+      <c r="B8" t="s">
+        <v>598</v>
+      </c>
+      <c r="C8" t="s">
+        <v>582</v>
+      </c>
+      <c r="D8" t="s">
+        <v>583</v>
+      </c>
+      <c r="E8" t="s">
+        <v>599</v>
+      </c>
+      <c r="F8" t="s">
+        <v>600</v>
+      </c>
+      <c r="J8">
+        <v>2</v>
+      </c>
+      <c r="K8" s="25">
+        <v>46233</v>
+      </c>
+      <c r="L8" t="s">
+        <v>587</v>
+      </c>
+      <c r="M8" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>601</v>
+      </c>
+      <c r="B9" t="s">
+        <v>598</v>
+      </c>
+      <c r="C9" t="s">
+        <v>582</v>
+      </c>
+      <c r="D9" t="s">
+        <v>583</v>
+      </c>
+      <c r="E9" t="s">
+        <v>584</v>
+      </c>
+      <c r="F9" t="s">
+        <v>602</v>
+      </c>
+      <c r="G9" t="s">
+        <v>603</v>
+      </c>
+      <c r="J9">
+        <v>3</v>
+      </c>
+      <c r="K9" s="25">
+        <v>46233</v>
+      </c>
+      <c r="L9" t="s">
+        <v>587</v>
+      </c>
+      <c r="M9" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>604</v>
+      </c>
+      <c r="B10" t="s">
+        <v>605</v>
+      </c>
+      <c r="C10" t="s">
+        <v>606</v>
+      </c>
+      <c r="D10" t="s">
+        <v>583</v>
+      </c>
+      <c r="E10" t="s">
+        <v>584</v>
+      </c>
+      <c r="F10" t="s">
+        <v>607</v>
+      </c>
+      <c r="G10" t="s">
+        <v>608</v>
+      </c>
+      <c r="J10">
+        <v>3</v>
+      </c>
+      <c r="K10" s="25">
+        <v>46233</v>
+      </c>
+      <c r="L10" t="s">
+        <v>587</v>
+      </c>
+      <c r="M10" t="s">
+        <v>609</v>
+      </c>
+    </row>
     <row r="307" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A307" s="3" t="s">
         <v>435</v>

</xml_diff>